<commit_message>
Deploy: latest leaderboard and meta to site
</commit_message>
<xml_diff>
--- a/ipl_fantasy_ledger.xlsx
+++ b/ipl_fantasy_ledger.xlsx
@@ -496,7 +496,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -677,7 +677,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -1325,7 +1325,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -1973,7 +1973,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H421"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -17159,7 +17159,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H133"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -21713,7 +21713,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -24371,7 +24371,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -25019,7 +25019,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -25667,7 +25667,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -26265,7 +26265,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -26813,7 +26813,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>

</xml_diff>